<commit_message>
105th Commit: Epic Three,Four And Six Completed
</commit_message>
<xml_diff>
--- a/EPIC_0003_Customer_Onboarding.xlsx
+++ b/EPIC_0003_Customer_Onboarding.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30131"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30228"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\EIT_PROJECTS\ABCD_Framework_For_WE1_Automation\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A491869D-541E-4D4B-9156-8D7218BB637B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C1CB0D88-DB3F-42FB-8FB6-B728F731BAE9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -320,6 +320,30 @@
   </si>
   <si>
     <t>This test case validates the end-to-end customer lifecycle including registration, admin verification, profile management, self-initiated account deletion, and post-deletion record verification. It covers initial customer onboarding via the mobile app using a random mobile number and OTP, updating and verifying customer details (name, email, emergency contact, gender, and profile photo) through the Super Admin portal under non-verified customers, confirming the customer's transition to the verified list, re-authenticating in the app to access profile settings, triggering account deletion under manage account options, and finally confirming that the deleted customer record accurately moves to the deleted customers section within the admin web panel.</t>
+  </si>
+  <si>
+    <t>1. Open the Customer Mobile App.
+2. Tap "Get Started" on the initial onboarding screen.
+3. Tap "Allow" on the system permission popup.
+4. Tap "Next" on the onboarding screen.
+5. Tap the Mobile Number input field.
+6. Dismiss/close any system auto-fill or phone number selector dialogs.
+7. Enter a new random Mobile Number.
+8. Tap "Continue" to proceed to OTP verification.
+9. Enter the verification OTP (123456).
+10. Confirm reaching the Registration page.
+11. Type the Customer Name into the name input field.
+12. Type the Email Address into the email input field.
+13. Select "Male" gender option.
+14. Select the agreement checkbox.
+15. Tap the "Sign Up" button.
+16. Tap "Allow" on the location permission prompt.
+17. Switch to the Super Admin Web Portal.
+18. Click the Dashboard Icon on the sidebar menu.
+19. Click the Customer Menu icon.
+20. Click the "Verified Customers" sub-menu link.
+21. Type the registered Customer Name into the filter input field.
+22. Verify that the customer is successfully listed in the Verified Customers grid view.</t>
   </si>
   <si>
     <t>1.Reload User App Completely,reload_app,user,
@@ -347,35 +371,11 @@
 23.Click Dashboard Icon,click,, "web.global.menu.dashboard"
 24. Click Customer Menu,click,,"admin.menu.customer_icon"
 25. Click Verified Customers Menu,click,,"admin.menu.verified_customers"
-27.Wait For Customer Filter,wait,3000,
-28. Enter Customer Name,type,{customerName},"admin.customer.filter_name"
-29.Wait For Customer,wait,2000,
-30. Verify Customer Available In Verified Customer List,verify,,"admin.customer.verified_list_heading"
-31.Wait For Data,wait,5000,</t>
-  </si>
-  <si>
-    <t>1. Open the Customer Mobile App.
-2. Tap "Get Started" on the initial onboarding screen.
-3. Tap "Allow" on the system permission popup.
-4. Tap "Next" on the onboarding screen.
-5. Tap the Mobile Number input field.
-6. Dismiss/close any system auto-fill or phone number selector dialogs.
-7. Enter a new random Mobile Number.
-8. Tap "Continue" to proceed to OTP verification.
-9. Enter the verification OTP (123456).
-10. Confirm reaching the Registration page.
-11. Type the Customer Name into the name input field.
-12. Type the Email Address into the email input field.
-13. Select "Male" gender option.
-14. Select the agreement checkbox.
-15. Tap the "Sign Up" button.
-16. Tap "Allow" on the location permission prompt.
-17. Switch to the Super Admin Web Portal.
-18. Click the Dashboard Icon on the sidebar menu.
-19. Click the Customer Menu icon.
-20. Click the "Verified Customers" sub-menu link.
-21. Type the registered Customer Name into the filter input field.
-22. Verify that the customer is successfully listed in the Verified Customers grid view.</t>
+26.Wait For Customer Filter,wait,3000,
+27. Enter Customer Name,type,{customerName},"admin.customer.filter_name"
+28.Wait For Customer,wait,2000,
+29. Verify Customer Available In Verified Customer List,verify,,"admin.customer.verified_list_heading"
+30.Wait For Data,wait,5000,</t>
   </si>
 </sst>
 </file>
@@ -883,10 +883,10 @@
         <v>27</v>
       </c>
       <c r="F2" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="G2" s="2" t="s">
         <v>29</v>
-      </c>
-      <c r="G2" s="2" t="s">
-        <v>28</v>
       </c>
       <c r="H2" s="2" t="s">
         <v>10</v>

</xml_diff>